<commit_message>
add all to repo
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2487721\IdeaProjects\BookingCab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{101541A2-6045-4522-AE0C-72A074A540C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DF9226-47B2-486F-A665-A975AF83F3A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5F60D20A-8113-4B45-AF7D-4A14A255CAA5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,18 +39,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>FromCity</t>
-  </si>
-  <si>
-    <t>ToCity</t>
-  </si>
-  <si>
-    <t>Delhi</t>
-  </si>
-  <si>
-    <t>Manali</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>SenderName</t>
+  </si>
+  <si>
+    <t>SenderEmail</t>
+  </si>
+  <si>
+    <t>SenderMobile</t>
+  </si>
+  <si>
+    <t>ReceiverName</t>
+  </si>
+  <si>
+    <t>ReceiverEmail</t>
+  </si>
+  <si>
+    <t>ReceiverMobile</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>TestUser</t>
+  </si>
+  <si>
+    <t>invalidemail.com</t>
+  </si>
+  <si>
+    <t>Receiver</t>
+  </si>
+  <si>
+    <t>receiver@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -120,13 +144,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -461,29 +491,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15EAA220-26E4-423E-9C4C-D2994CACC4C9}">
-  <dimension ref="A1:B2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{934637D7-41E9-41E1-8664-0770E40A20EE}">
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.08984375" customWidth="1"/>
-    <col min="2" max="2" width="28.1796875" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="14.6328125" customWidth="1"/>
+    <col min="3" max="3" width="20.26953125" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" customWidth="1"/>
+    <col min="5" max="5" width="24.6328125" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="13.26953125" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2"/>
     </row>
-    <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3">
+        <v>9999999999</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="3">
+        <v>8888888888</v>
+      </c>
+      <c r="G2" s="3">
+        <v>500</v>
+      </c>
+      <c r="H2" s="4">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="I2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>